<commit_message>
Atualiza pacote mensal da indústria CVM em 10/10/2026
</commit_message>
<xml_diff>
--- a/data/industry_study/generated_revision/top100_fidcs_middle_market.xlsx
+++ b/data/industry_study/generated_revision/top100_fidcs_middle_market.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Leia-me" sheetId="1" r:id="R94c6953f19e74020"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Top 100 FIDCs" sheetId="2" r:id="R7fb71cc8fb0a461f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Leia-me" sheetId="1" r:id="R264c4324ac4d4d2f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Top 100 FIDCs" sheetId="2" r:id="Rf8e2aecf45c2441f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -890,7 +890,7 @@
         <x:v>58815322507.62</x:v>
       </x:c>
       <x:c r="H5" s="49" t="n">
-        <x:v>0.06965301206862962</x:v>
+        <x:v>0.06965277452767916</x:v>
       </x:c>
       <x:c r="I5" s="49" t="n">
         <x:v>0.0012711173696075</x:v>
@@ -1015,7 +1015,7 @@
         <x:v>33455157284.84</x:v>
       </x:c>
       <x:c r="H6" s="50" t="n">
-        <x:v>0.03961981971308513</x:v>
+        <x:v>0.03961968459574631</x:v>
       </x:c>
       <x:c r="I6" s="50" t="n">
         <x:v>1</x:v>
@@ -1140,7 +1140,7 @@
         <x:v>20198291907.77</x:v>
       </x:c>
       <x:c r="H7" s="51" t="n">
-        <x:v>0.023920159067993482</x:v>
+        <x:v>0.023920077491947432</x:v>
       </x:c>
       <x:c r="I7" s="51" t="n">
         <x:v>0</x:v>
@@ -1265,7 +1265,7 @@
         <x:v>10699481597.570002</x:v>
       </x:c>
       <x:c r="H8" s="50" t="n">
-        <x:v>0.012671036884088674</x:v>
+        <x:v>0.012670993671454283</x:v>
       </x:c>
       <x:c r="I8" s="50" t="n">
         <x:v>0.0326072904035432</x:v>
@@ -1390,7 +1390,7 @@
         <x:v>10070614364.8</x:v>
       </x:c>
       <x:c r="H9" s="51" t="n">
-        <x:v>0.011926290530822998</x:v>
+        <x:v>0.011926249858032202</x:v>
       </x:c>
       <x:c r="I9" s="51" t="n">
         <x:v>0.1603537622701268</x:v>
@@ -1515,7 +1515,7 @@
         <x:v>8932735715.03</x:v>
       </x:c>
       <x:c r="H10" s="50" t="n">
-        <x:v>0.010578739043456804</x:v>
+        <x:v>0.010578702966284369</x:v>
       </x:c>
       <x:c r="I10" s="50" t="n">
         <x:v>0</x:v>
@@ -1640,7 +1640,7 @@
         <x:v>8239227134.05</x:v>
       </x:c>
       <x:c r="H11" s="51" t="n">
-        <x:v>0.009757440111457582</x:v>
+        <x:v>0.009757406835199609</x:v>
       </x:c>
       <x:c r="I11" s="51" t="n">
         <x:v>0</x:v>
@@ -1765,7 +1765,7 @@
         <x:v>7959831126.05</x:v>
       </x:c>
       <x:c r="H12" s="50" t="n">
-        <x:v>0.009426560798254298</x:v>
+        <x:v>0.009426528650409645</x:v>
       </x:c>
       <x:c r="I12" s="50" t="n">
         <x:v>0.1110477241038992</x:v>
@@ -1890,7 +1890,7 @@
         <x:v>7174237038.23</x:v>
       </x:c>
       <x:c r="H13" s="51" t="n">
-        <x:v>0.008496208091731584</x:v>
+        <x:v>0.008496179116712622</x:v>
       </x:c>
       <x:c r="I13" s="51" t="n">
         <x:v>0.7364651414444897</x:v>
@@ -2015,7 +2015,7 @@
         <x:v>6705565454.97</x:v>
       </x:c>
       <x:c r="H14" s="50" t="n">
-        <x:v>0.007941176068557636</x:v>
+        <x:v>0.007941148986390548</x:v>
       </x:c>
       <x:c r="I14" s="50" t="n">
         <x:v>0.84310494226191</x:v>
@@ -2140,7 +2140,7 @@
         <x:v>6476101048.84</x:v>
       </x:c>
       <x:c r="H15" s="51" t="n">
-        <x:v>0.007669429075290311</x:v>
+        <x:v>0.007669402919874803</x:v>
       </x:c>
       <x:c r="I15" s="51" t="n">
         <x:v>1</x:v>
@@ -2265,7 +2265,7 @@
         <x:v>6460522602.03</x:v>
       </x:c>
       <x:c r="H16" s="50" t="n">
-        <x:v>0.007650980043687587</x:v>
+        <x:v>0.007650953951189681</x:v>
       </x:c>
       <x:c r="I16" s="50" t="n">
         <x:v>1</x:v>
@@ -2390,7 +2390,7 @@
         <x:v>6390290390.09</x:v>
       </x:c>
       <x:c r="H17" s="51" t="n">
-        <x:v>0.007567806392718836</x:v>
+        <x:v>0.007567780583871952</x:v>
       </x:c>
       <x:c r="I17" s="51" t="n">
         <x:v>0</x:v>
@@ -2515,7 +2515,7 @@
         <x:v>6111960853.79</x:v>
       </x:c>
       <x:c r="H18" s="50" t="n">
-        <x:v>0.007238190066149372</x:v>
+        <x:v>0.007238165381408586</x:v>
       </x:c>
       <x:c r="I18" s="50" t="n">
         <x:v>0</x:v>
@@ -2640,7 +2640,7 @@
         <x:v>5933688515.09</x:v>
       </x:c>
       <x:c r="H19" s="51" t="n">
-        <x:v>0.0070270681198680235</x:v>
+        <x:v>0.007027044155126363</x:v>
       </x:c>
       <x:c r="I19" s="51" t="n">
         <x:v>0</x:v>
@@ -2765,7 +2765,7 @@
         <x:v>4985976955.36</x:v>
       </x:c>
       <x:c r="H20" s="50" t="n">
-        <x:v>0.005904725133499101</x:v>
+        <x:v>0.005904704996336633</x:v>
       </x:c>
       <x:c r="I20" s="50" t="n">
         <x:v>1</x:v>
@@ -2890,7 +2890,7 @@
         <x:v>4670319122.88</x:v>
       </x:c>
       <x:c r="H21" s="51" t="n">
-        <x:v>0.005530902158840782</x:v>
+        <x:v>0.005530883296544427</x:v>
       </x:c>
       <x:c r="I21" s="51" t="n">
         <x:v>0.1272759196611239</x:v>
@@ -3015,7 +3015,7 @@
         <x:v>4584487367.37</x:v>
       </x:c>
       <x:c r="H22" s="50" t="n">
-        <x:v>0.005429254492084638</x:v>
+        <x:v>0.005429235976442112</x:v>
       </x:c>
       <x:c r="I22" s="50" t="n">
         <x:v>0</x:v>
@@ -3140,7 +3140,7 @@
         <x:v>4231296076.69</x:v>
       </x:c>
       <x:c r="H23" s="51" t="n">
-        <x:v>0.0050109819028442805</x:v>
+        <x:v>0.005010964813656483</x:v>
       </x:c>
       <x:c r="I23" s="51" t="n">
         <x:v>1</x:v>
@@ -3265,7 +3265,7 @@
         <x:v>3772944315.34</x:v>
       </x:c>
       <x:c r="H24" s="50" t="n">
-        <x:v>0.004468171298331265</x:v>
+        <x:v>0.0044681560603160595</x:v>
       </x:c>
       <x:c r="I24" s="50" t="n">
         <x:v>0.7056380854286087</x:v>
@@ -3390,7 +3390,7 @@
         <x:v>3771058923.75</x:v>
       </x:c>
       <x:c r="H25" s="51" t="n">
-        <x:v>0.004465938492362117</x:v>
+        <x:v>0.004465923261961555</x:v>
       </x:c>
       <x:c r="I25" s="51" t="n">
         <x:v>0.0303918848813086</x:v>
@@ -3515,7 +3515,7 @@
         <x:v>3765650088.95</x:v>
       </x:c>
       <x:c r="H26" s="50" t="n">
-        <x:v>0.0044595329908781655</x:v>
+        <x:v>0.0044595177823225874</x:v>
       </x:c>
       <x:c r="I26" s="50" t="n">
         <x:v>1</x:v>
@@ -3640,7 +3640,7 @@
         <x:v>3686239660.81</x:v>
       </x:c>
       <x:c r="H27" s="51" t="n">
-        <x:v>0.0043654898865681645</x:v>
+        <x:v>0.004365474998732218</x:v>
       </x:c>
       <x:c r="I27" s="51" t="n">
         <x:v>0</x:v>
@@ -3765,7 +3765,7 @@
         <x:v>3658919018.85</x:v>
       </x:c>
       <x:c r="H28" s="50" t="n">
-        <x:v>0.0043331349674241605</x:v>
+        <x:v>0.00433312018992972</x:v>
       </x:c>
       <x:c r="I28" s="50" t="n">
         <x:v>0</x:v>
@@ -3890,7 +3890,7 @@
         <x:v>3599560973.43</x:v>
       </x:c>
       <x:c r="H29" s="51" t="n">
-        <x:v>0.004262839226829116</x:v>
+        <x:v>0.004262824689067553</x:v>
       </x:c>
       <x:c r="I29" s="51" t="n">
         <x:v>1</x:v>
@@ -4015,7 +4015,7 @@
         <x:v>3389462172.19</x:v>
       </x:c>
       <x:c r="H30" s="50" t="n">
-        <x:v>0.004014026269347188</x:v>
+        <x:v>0.004014012580124183</x:v>
       </x:c>
       <x:c r="I30" s="50" t="n">
         <x:v>0.0534980276932435</x:v>
@@ -4140,7 +4140,7 @@
         <x:v>3371226156.53</x:v>
       </x:c>
       <x:c r="H31" s="51" t="n">
-        <x:v>0.003992429968167592</x:v>
+        <x:v>0.0039924163525954705</x:v>
       </x:c>
       <x:c r="I31" s="51" t="n">
         <x:v>0</x:v>
@@ -4265,7 +4265,7 @@
         <x:v>3334605706.65</x:v>
       </x:c>
       <x:c r="H32" s="50" t="n">
-        <x:v>0.003949061598690066</x:v>
+        <x:v>0.003949048131019139</x:v>
       </x:c>
       <x:c r="I32" s="50" t="n">
         <x:v>0.4811159979432757</x:v>
@@ -4390,7 +4390,7 @@
         <x:v>3311135945.94</x:v>
       </x:c>
       <x:c r="H33" s="51" t="n">
-        <x:v>0.003921267148939838</x:v>
+        <x:v>0.003921253776057634</x:v>
       </x:c>
       <x:c r="I33" s="51" t="n">
         <x:v>0.7289331396097506</x:v>
@@ -4515,7 +4515,7 @@
         <x:v>3256435200.06</x:v>
       </x:c>
       <x:c r="H34" s="50" t="n">
-        <x:v>0.0038564868918486853</x:v>
+        <x:v>0.0038564737398896457</x:v>
       </x:c>
       <x:c r="I34" s="50" t="n">
         <x:v>0.1617789634703957</x:v>
@@ -4640,7 +4640,7 @@
         <x:v>3196029095.69</x:v>
       </x:c>
       <x:c r="H35" s="51" t="n">
-        <x:v>0.0037849499702215465</x:v>
+        <x:v>0.003784937062228243</x:v>
       </x:c>
       <x:c r="I35" s="51" t="n">
         <x:v>0</x:v>
@@ -4765,7 +4765,7 @@
         <x:v>3141061787.79</x:v>
       </x:c>
       <x:c r="H36" s="50" t="n">
-        <x:v>0.0037198540326783534</x:v>
+        <x:v>0.0037198413466847944</x:v>
       </x:c>
       <x:c r="I36" s="50" t="n">
         <x:v>1</x:v>
@@ -4890,7 +4890,7 @@
         <x:v>3100556826.01</x:v>
       </x:c>
       <x:c r="H37" s="51" t="n">
-        <x:v>0.003671885366157207</x:v>
+        <x:v>0.0036718728437534526</x:v>
       </x:c>
       <x:c r="I37" s="51" t="n">
         <x:v>0.1896520557500736</x:v>
@@ -5015,7 +5015,7 @@
         <x:v>3091810070.76</x:v>
       </x:c>
       <x:c r="H38" s="50" t="n">
-        <x:v>0.0036615268775352892</x:v>
+        <x:v>0.0036615143904575767</x:v>
       </x:c>
       <x:c r="I38" s="50" t="n">
         <x:v>0</x:v>
@@ -5140,7 +5140,7 @@
         <x:v>3058103926.17</x:v>
       </x:c>
       <x:c r="H39" s="51" t="n">
-        <x:v>0.00362160982198212</x:v>
+        <x:v>0.003621597471035423</x:v>
       </x:c>
       <x:c r="I39" s="51" t="n">
         <x:v>0</x:v>
@@ -5265,7 +5265,7 @@
         <x:v>3000510455.02</x:v>
       </x:c>
       <x:c r="H40" s="50" t="n">
-        <x:v>0.003553403807459875</x:v>
+        <x:v>0.0035533916891193652</x:v>
       </x:c>
       <x:c r="I40" s="50" t="n">
         <x:v>0</x:v>
@@ -5390,7 +5390,7 @@
         <x:v>2966345679.42</x:v>
       </x:c>
       <x:c r="H41" s="51" t="n">
-        <x:v>0.003512943610597391</x:v>
+        <x:v>0.0035129316302401977</x:v>
       </x:c>
       <x:c r="I41" s="51" t="n">
         <x:v>0.1524969562841521</x:v>
@@ -5515,7 +5515,7 @@
         <x:v>2940889060.03</x:v>
       </x:c>
       <x:c r="H42" s="50" t="n">
-        <x:v>0.003482796190809487</x:v>
+        <x:v>0.0034827843132654605</x:v>
       </x:c>
       <x:c r="I42" s="50" t="n">
         <x:v>0</x:v>
@@ -5640,7 +5640,7 @@
         <x:v>2758097886.13</x:v>
       </x:c>
       <x:c r="H43" s="51" t="n">
-        <x:v>0.0032663227396939865</x:v>
+        <x:v>0.0032663116003995747</x:v>
       </x:c>
       <x:c r="I43" s="51" t="n">
         <x:v>1</x:v>
@@ -5765,7 +5765,7 @@
         <x:v>2703044510.17</x:v>
       </x:c>
       <x:c r="H44" s="50" t="n">
-        <x:v>0.003201124874636562</x:v>
+        <x:v>0.003201113957689503</x:v>
       </x:c>
       <x:c r="I44" s="50" t="n">
         <x:v>0.1623408260106682</x:v>
@@ -5890,7 +5890,7 @@
         <x:v>2661374071.86</x:v>
       </x:c>
       <x:c r="H45" s="51" t="n">
-        <x:v>0.003151775973384929</x:v>
+        <x:v>0.0031517652247347538</x:v>
       </x:c>
       <x:c r="I45" s="51" t="n">
         <x:v>0.6957359372662582</x:v>
@@ -6015,7 +6015,7 @@
         <x:v>2641955191.86</x:v>
       </x:c>
       <x:c r="H46" s="50" t="n">
-        <x:v>0.003128778845675155</x:v>
+        <x:v>0.003128768175453169</x:v>
       </x:c>
       <x:c r="I46" s="50" t="n">
         <x:v>0.3493155766177357</x:v>
@@ -6140,7 +6140,7 @@
         <x:v>2579461850.15</x:v>
       </x:c>
       <x:c r="H47" s="51" t="n">
-        <x:v>0.0030547700789329223</x:v>
+        <x:v>0.003054759661106522</x:v>
       </x:c>
       <x:c r="I47" s="51" t="n">
         <x:v>0.4829575505614513</x:v>
@@ -6265,7 +6265,7 @@
         <x:v>2575168330.09</x:v>
       </x:c>
       <x:c r="H48" s="50" t="n">
-        <x:v>0.003049685407255447</x:v>
+        <x:v>0.0030496750067695423</x:v>
       </x:c>
       <x:c r="I48" s="50" t="n">
         <x:v>0.0876860137103579</x:v>
@@ -6390,7 +6390,7 @@
         <x:v>2567223636.65</x:v>
       </x:c>
       <x:c r="H49" s="51" t="n">
-        <x:v>0.0030402767735106234</x:v>
+        <x:v>0.0030402664051114255</x:v>
       </x:c>
       <x:c r="I49" s="51" t="n">
         <x:v>1</x:v>
@@ -6515,7 +6515,7 @@
         <x:v>2543457792.98</x:v>
       </x:c>
       <x:c r="H50" s="50" t="n">
-        <x:v>0.0030121316826501043</x:v>
+        <x:v>0.003012121410235437</x:v>
       </x:c>
       <x:c r="I50" s="50" t="n">
         <x:v>0.0760103608607955</x:v>
@@ -6640,7 +6640,7 @@
         <x:v>2539517617.4</x:v>
       </x:c>
       <x:c r="H51" s="51" t="n">
-        <x:v>0.003007465464978839</x:v>
+        <x:v>0.0030074552084775933</x:v>
       </x:c>
       <x:c r="I51" s="51" t="n">
         <x:v>0</x:v>
@@ -6765,7 +6765,7 @@
         <x:v>2531012852.93</x:v>
       </x:c>
       <x:c r="H52" s="50" t="n">
-        <x:v>0.002997393557914263</x:v>
+        <x:v>0.002997383335761717</x:v>
       </x:c>
       <x:c r="I52" s="50" t="n">
         <x:v>0</x:v>
@@ -6890,7 +6890,7 @@
         <x:v>2498979874.47</x:v>
       </x:c>
       <x:c r="H53" s="51" t="n">
-        <x:v>0.00295945797684218</x:v>
+        <x:v>0.0029594478840631344</x:v>
       </x:c>
       <x:c r="I53" s="51" t="n">
         <x:v>0.2593848573902249</x:v>
@@ -7015,7 +7015,7 @@
         <x:v>2464338064.69</x:v>
       </x:c>
       <x:c r="H54" s="50" t="n">
-        <x:v>0.0029184328444139276</x:v>
+        <x:v>0.002918422891544825</x:v>
       </x:c>
       <x:c r="I54" s="50" t="n">
         <x:v>0.180905841005734</x:v>
@@ -7140,7 +7140,7 @@
         <x:v>2420168048.15</x:v>
       </x:c>
       <x:c r="H55" s="51" t="n">
-        <x:v>0.002866123776573084</x:v>
+        <x:v>0.0028661140020960615</x:v>
       </x:c>
       <x:c r="I55" s="51" t="n">
         <x:v>0</x:v>
@@ -7265,7 +7265,7 @@
         <x:v>2402205778.31</x:v>
       </x:c>
       <x:c r="H56" s="50" t="n">
-        <x:v>0.0028448516633787133</x:v>
+        <x:v>0.002844841961446981</x:v>
       </x:c>
       <x:c r="I56" s="50" t="n">
         <x:v>0.0864587494545391</x:v>
@@ -7390,7 +7390,7 @@
         <x:v>2373894609.18</x:v>
       </x:c>
       <x:c r="H57" s="51" t="n">
-        <x:v>0.0028113236961583785</x:v>
+        <x:v>0.0028113141085686533</x:v>
       </x:c>
       <x:c r="I57" s="51" t="n">
         <x:v>0.1527059368171675</x:v>
@@ -7515,7 +7515,7 @@
         <x:v>2373588339.88</x:v>
       </x:c>
       <x:c r="H58" s="50" t="n">
-        <x:v>0.002810960991707572</x:v>
+        <x:v>0.0028109514053547948</x:v>
       </x:c>
       <x:c r="I58" s="50" t="n">
         <x:v>1</x:v>
@@ -7640,7 +7640,7 @@
         <x:v>2234066329.65</x:v>
       </x:c>
       <x:c r="H59" s="51" t="n">
-        <x:v>0.0026457297586197893</x:v>
+        <x:v>0.0026457207357628754</x:v>
       </x:c>
       <x:c r="I59" s="51" t="n">
         <x:v>0.1327136681119272</x:v>
@@ -7765,7 +7765,7 @@
         <x:v>2220692700.39</x:v>
       </x:c>
       <x:c r="H60" s="50" t="n">
-        <x:v>0.0026298918184278013</x:v>
+        <x:v>0.0026298828495837615</x:v>
       </x:c>
       <x:c r="I60" s="50" t="n">
         <x:v>0</x:v>
@@ -7890,7 +7890,7 @@
         <x:v>2207595143.13</x:v>
       </x:c>
       <x:c r="H61" s="51" t="n">
-        <x:v>0.002614380821037927</x:v>
+        <x:v>0.0026143719050917722</x:v>
       </x:c>
       <x:c r="I61" s="51" t="n">
         <x:v>0</x:v>
@@ -8015,7 +8015,7 @@
         <x:v>2162550453.27</x:v>
       </x:c>
       <x:c r="H62" s="50" t="n">
-        <x:v>0.002561035906946199</x:v>
+        <x:v>0.0025610271729247197</x:v>
       </x:c>
       <x:c r="I62" s="50" t="n">
         <x:v>0.4168932745358105</x:v>
@@ -8140,7 +8140,7 @@
         <x:v>2125721812.65</x:v>
       </x:c>
       <x:c r="H63" s="51" t="n">
-        <x:v>0.002517420984164066</x:v>
+        <x:v>0.002517412398884614</x:v>
       </x:c>
       <x:c r="I63" s="51" t="n">
         <x:v>0.1507558774200163</x:v>
@@ -8265,7 +8265,7 @@
         <x:v>2090403784.62</x:v>
       </x:c>
       <x:c r="H64" s="50" t="n">
-        <x:v>0.0024755950291623727</x:v>
+        <x:v>0.0024755865865239467</x:v>
       </x:c>
       <x:c r="I64" s="50" t="n">
         <x:v>0.4527500152326454</x:v>
@@ -8390,7 +8390,7 @@
         <x:v>2082486408.15</x:v>
       </x:c>
       <x:c r="H65" s="51" t="n">
-        <x:v>0.0024662187459881142</x:v>
+        <x:v>0.0024662103353260685</x:v>
       </x:c>
       <x:c r="I65" s="51" t="n">
         <x:v>0</x:v>
@@ -8515,7 +8515,7 @@
         <x:v>2045856427.66</x:v>
       </x:c>
       <x:c r="H66" s="50" t="n">
-        <x:v>0.0024228390897290996</x:v>
+        <x:v>0.002422830827006741</x:v>
       </x:c>
       <x:c r="I66" s="50" t="n">
         <x:v>0.0393499895555923</x:v>
@@ -8640,7 +8640,7 @@
         <x:v>2040649598.42</x:v>
       </x:c>
       <x:c r="H67" s="51" t="n">
-        <x:v>0.0024166728166487125</x:v>
+        <x:v>0.0024166645749554854</x:v>
       </x:c>
       <x:c r="I67" s="51" t="n">
         <x:v>0</x:v>
@@ -8765,7 +8765,7 @@
         <x:v>2040580910.81</x:v>
       </x:c>
       <x:c r="H68" s="50" t="n">
-        <x:v>0.0024165914722179705</x:v>
+        <x:v>0.002416583230802156</x:v>
       </x:c>
       <x:c r="I68" s="50" t="n">
         <x:v>0</x:v>
@@ -8890,7 +8890,7 @@
         <x:v>1999981369.56</x:v>
       </x:c>
       <x:c r="H69" s="51" t="n">
-        <x:v>0.0023685107984054497</x:v>
+        <x:v>0.002368502720961424</x:v>
       </x:c>
       <x:c r="I69" s="51" t="n">
         <x:v>0.0930889101736938</x:v>
@@ -9015,7 +9015,7 @@
         <x:v>1960417320.47</x:v>
       </x:c>
       <x:c r="H70" s="50" t="n">
-        <x:v>0.0023216564231974828</x:v>
+        <x:v>0.002321648505543141</x:v>
       </x:c>
       <x:c r="I70" s="50" t="n">
         <x:v>0</x:v>
@@ -9140,7 +9140,7 @@
         <x:v>1944596528.21</x:v>
       </x:c>
       <x:c r="H71" s="51" t="n">
-        <x:v>0.002302920390013642</x:v>
+        <x:v>0.0023029125362556777</x:v>
       </x:c>
       <x:c r="I71" s="51" t="n">
         <x:v>1</x:v>
@@ -9265,7 +9265,7 @@
         <x:v>1927443335.68</x:v>
       </x:c>
       <x:c r="H72" s="50" t="n">
-        <x:v>0.0022826064399175117</x:v>
+        <x:v>0.0022825986554371688</x:v>
       </x:c>
       <x:c r="I72" s="50" t="n">
         <x:v>0</x:v>
@@ -9390,7 +9390,7 @@
         <x:v>1925682597.46</x:v>
       </x:c>
       <x:c r="H73" s="51" t="n">
-        <x:v>0.002280521256749954</x:v>
+        <x:v>0.0022805134793808094</x:v>
       </x:c>
       <x:c r="I73" s="51" t="n">
         <x:v>0.1027449904369085</x:v>
@@ -9515,7 +9515,7 @@
         <x:v>1925498329.61</x:v>
       </x:c>
       <x:c r="H74" s="50" t="n">
-        <x:v>0.0022803030345209035</x:v>
+        <x:v>0.002280295257895973</x:v>
       </x:c>
       <x:c r="I74" s="50" t="n">
         <x:v>0.1153248886507287</x:v>
@@ -9640,7 +9640,7 @@
         <x:v>1924331624.55</x:v>
       </x:c>
       <x:c r="H75" s="51" t="n">
-        <x:v>0.0022789213448835785</x:v>
+        <x:v>0.002278913572970689</x:v>
       </x:c>
       <x:c r="I75" s="51" t="n">
         <x:v>0.3851477559871331</x:v>
@@ -9765,7 +9765,7 @@
         <x:v>1919387163.23</x:v>
       </x:c>
       <x:c r="H76" s="50" t="n">
-        <x:v>0.0022730657853233943</x:v>
+        <x:v>0.0022730580333799955</x:v>
       </x:c>
       <x:c r="I76" s="50" t="n">
         <x:v>1</x:v>
@@ -9890,7 +9890,7 @@
         <x:v>1911439961.8</x:v>
       </x:c>
       <x:c r="H77" s="51" t="n">
-        <x:v>0.002263654181450204</x:v>
+        <x:v>0.0022636464616036423</x:v>
       </x:c>
       <x:c r="I77" s="51" t="n">
         <x:v>0.3289671657228036</x:v>
@@ -10015,7 +10015,7 @@
         <x:v>1911426358.03</x:v>
       </x:c>
       <x:c r="H78" s="50" t="n">
-        <x:v>0.0022636380709620597</x:v>
+        <x:v>0.0022636303511704395</x:v>
       </x:c>
       <x:c r="I78" s="50" t="n">
         <x:v>0.4739448173839156</x:v>
@@ -10140,7 +10140,7 @@
         <x:v>1897667543.94</x:v>
       </x:c>
       <x:c r="H79" s="51" t="n">
-        <x:v>0.0022473439693062093</x:v>
+        <x:v>0.0022473363050831323</x:v>
       </x:c>
       <x:c r="I79" s="51" t="n">
         <x:v>0.8815886150370092</x:v>
@@ -10265,7 +10265,7 @@
         <x:v>1866969812.56</x:v>
       </x:c>
       <x:c r="H80" s="50" t="n">
-        <x:v>0.002210989676527934</x:v>
+        <x:v>0.0022109821362856154</x:v>
       </x:c>
       <x:c r="I80" s="50" t="n">
         <x:v>0</x:v>
@@ -10390,7 +10390,7 @@
         <x:v>1855894253.21</x:v>
       </x:c>
       <x:c r="H81" s="51" t="n">
-        <x:v>0.002197873263386232</x:v>
+        <x:v>0.0021978657678754358</x:v>
       </x:c>
       <x:c r="I81" s="51" t="n">
         <x:v>0.1873702924545502</x:v>
@@ -10515,7 +10515,7 @@
         <x:v>1847170248.89</x:v>
       </x:c>
       <x:c r="H82" s="50" t="n">
-        <x:v>0.0021875417179269855</x:v>
+        <x:v>0.0021875342576503456</x:v>
       </x:c>
       <x:c r="I82" s="50" t="n">
         <x:v>0.3460699773697318</x:v>
@@ -10640,7 +10640,7 @@
         <x:v>1800909934.43</x:v>
       </x:c>
       <x:c r="H83" s="51" t="n">
-        <x:v>0.0021327571804288952</x:v>
+        <x:v>0.002132749906986546</x:v>
       </x:c>
       <x:c r="I83" s="51" t="n">
         <x:v>0</x:v>
@@ -10765,7 +10765,7 @@
         <x:v>1755240553.43</x:v>
       </x:c>
       <x:c r="H84" s="50" t="n">
-        <x:v>0.0020786724655903815</x:v>
+        <x:v>0.0020786653765956847</x:v>
       </x:c>
       <x:c r="I84" s="50" t="n">
         <x:v>0</x:v>
@@ -10890,7 +10890,7 @@
         <x:v>1737053741.97</x:v>
       </x:c>
       <x:c r="H85" s="51" t="n">
-        <x:v>0.002057134435293104</x:v>
+        <x:v>0.002057127419750567</x:v>
       </x:c>
       <x:c r="I85" s="51" t="n">
         <x:v>1</x:v>
@@ -11015,7 +11015,7 @@
         <x:v>1717939470.45</x:v>
       </x:c>
       <x:c r="H86" s="50" t="n">
-        <x:v>0.0020344980451807632</x:v>
+        <x:v>0.0020344911068361747</x:v>
       </x:c>
       <x:c r="I86" s="50" t="n">
         <x:v>0</x:v>
@@ -11140,7 +11140,7 @@
         <x:v>1717932634.87</x:v>
       </x:c>
       <x:c r="H87" s="51" t="n">
-        <x:v>0.0020344899500328332</x:v>
+        <x:v>0.002034483011715852</x:v>
       </x:c>
       <x:c r="I87" s="51" t="n">
         <x:v>0.1505283858312573</x:v>
@@ -11265,7 +11265,7 @@
         <x:v>1695951362.31</x:v>
       </x:c>
       <x:c r="H88" s="50" t="n">
-        <x:v>0.0020084582668314505</x:v>
+        <x:v>0.0020084514172915456</x:v>
       </x:c>
       <x:c r="I88" s="50" t="n">
         <x:v>0.7583035475960594</x:v>
@@ -11390,7 +11390,7 @@
         <x:v>1626299680.36</x:v>
       </x:c>
       <x:c r="H89" s="51" t="n">
-        <x:v>0.0019259721180419891</x:v>
+        <x:v>0.0019259655498084858</x:v>
       </x:c>
       <x:c r="I89" s="51" t="n">
         <x:v>0.4183096467682989</x:v>
@@ -11515,7 +11515,7 @@
         <x:v>1596122150.92</x:v>
       </x:c>
       <x:c r="H90" s="50" t="n">
-        <x:v>0.001890233882958548</x:v>
+        <x:v>0.0018902274366048323</x:v>
       </x:c>
       <x:c r="I90" s="50" t="n">
         <x:v>0.7492493155245668</x:v>
@@ -11640,10 +11640,10 @@
         <x:v>1572064332.62</x:v>
       </x:c>
       <x:c r="H91" s="51" t="n">
-        <x:v>0.001861743016345044</x:v>
+        <x:v>0.001861736667155074</x:v>
       </x:c>
       <x:c r="I91" s="51" t="n">
-        <x:v>0.2179779669744</x:v>
+        <x:v>0.2032424948441643</x:v>
       </x:c>
       <x:c r="J91" s="51" t="str">
         <x:v>N/D</x:v>
@@ -11765,7 +11765,7 @@
         <x:v>1565448244.56</x:v>
       </x:c>
       <x:c r="H92" s="50" t="n">
-        <x:v>0.0018539078053516744</x:v>
+        <x:v>0.0018539014828824936</x:v>
       </x:c>
       <x:c r="I92" s="50" t="n">
         <x:v>0.2103059766797605</x:v>
@@ -11890,7 +11890,7 @@
         <x:v>1550515087.47</x:v>
       </x:c>
       <x:c r="H93" s="51" t="n">
-        <x:v>0.0018362229687025554</x:v>
+        <x:v>0.0018362167065448067</x:v>
       </x:c>
       <x:c r="I93" s="51" t="n">
         <x:v>0.2164128724195619</x:v>
@@ -12015,7 +12015,7 @@
         <x:v>1544332585.59</x:v>
       </x:c>
       <x:c r="H94" s="50" t="n">
-        <x:v>0.0018289012392670638</x:v>
+        <x:v>0.0018288950020789543</x:v>
       </x:c>
       <x:c r="I94" s="50" t="n">
         <x:v>0.2072216817801345</x:v>
@@ -12140,7 +12140,7 @@
         <x:v>1514334849.03</x:v>
       </x:c>
       <x:c r="H95" s="51" t="n">
-        <x:v>0.0017933759268559221</x:v>
+        <x:v>0.00179336981082146</x:v>
       </x:c>
       <x:c r="I95" s="51" t="n">
         <x:v>0.217904449537328</x:v>
@@ -12265,7 +12265,7 @@
         <x:v>1502648710.95</x:v>
       </x:c>
       <x:c r="H96" s="50" t="n">
-        <x:v>0.0017795364258208568</x:v>
+        <x:v>0.0017795303569838976</x:v>
       </x:c>
       <x:c r="I96" s="50" t="n">
         <x:v>0.150078915375806</x:v>
@@ -12390,7 +12390,7 @@
         <x:v>1498192276.83</x:v>
       </x:c>
       <x:c r="H97" s="51" t="n">
-        <x:v>0.0017742588204910008</x:v>
+        <x:v>0.0017742527696525078</x:v>
       </x:c>
       <x:c r="I97" s="51" t="n">
         <x:v>0</x:v>
@@ -12515,7 +12515,7 @@
         <x:v>1487482332.28</x:v>
       </x:c>
       <x:c r="H98" s="50" t="n">
-        <x:v>0.0017615753926835812</x:v>
+        <x:v>0.0017615693850999798</x:v>
       </x:c>
       <x:c r="I98" s="50" t="n">
         <x:v>0.4359813410538953</x:v>
@@ -12640,7 +12640,7 @@
         <x:v>1472677074.3</x:v>
       </x:c>
       <x:c r="H99" s="51" t="n">
-        <x:v>0.0017440420226569778</x:v>
+        <x:v>0.0017440360748682548</x:v>
       </x:c>
       <x:c r="I99" s="51" t="n">
         <x:v>0.1141825541295485</x:v>
@@ -12765,7 +12765,7 @@
         <x:v>1465748408.7</x:v>
       </x:c>
       <x:c r="H100" s="50" t="n">
-        <x:v>0.0017358366365759312</x:v>
+        <x:v>0.001735830716770423</x:v>
       </x:c>
       <x:c r="I100" s="50" t="n">
         <x:v>0</x:v>
@@ -12890,7 +12890,7 @@
         <x:v>1457599019.29</x:v>
       </x:c>
       <x:c r="H101" s="51" t="n">
-        <x:v>0.0017261855882652949</x:v>
+        <x:v>0.0017261797013732117</x:v>
       </x:c>
       <x:c r="I101" s="51" t="n">
         <x:v>0.0490927291065483</x:v>
@@ -13015,7 +13015,7 @@
         <x:v>1455000054.14</x:v>
       </x:c>
       <x:c r="H102" s="50" t="n">
-        <x:v>0.0017231077210830578</x:v>
+        <x:v>0.0017231018446875704</x:v>
       </x:c>
       <x:c r="I102" s="50" t="n">
         <x:v>0.1712974829590509</x:v>
@@ -13140,7 +13140,7 @@
         <x:v>1453818390.53</x:v>
       </x:c>
       <x:c r="H103" s="51" t="n">
-        <x:v>0.0017217083165371125</x:v>
+        <x:v>0.0017217024449140803</x:v>
       </x:c>
       <x:c r="I103" s="51" t="n">
         <x:v>0.1498724384837788</x:v>
@@ -13265,7 +13265,7 @@
         <x:v>1443190109.93</x:v>
       </x:c>
       <x:c r="H104" s="50" t="n">
-        <x:v>0.0017091216006042932</x:v>
+        <x:v>0.0017091157719063316</x:v>
       </x:c>
       <x:c r="I104" s="50" t="n">
         <x:v>0.7773601887411222</x:v>
@@ -13390,7 +13390,7 @@
         <x:v>790811150.71</x:v>
       </x:c>
       <x:c r="H105" s="51" t="n">
-        <x:v>0.0009365310989712611</x:v>
+        <x:v>0.0009365279050751068</x:v>
       </x:c>
       <x:c r="I105" s="51" t="n">
         <x:v>0.2027501641420936</x:v>
@@ -13515,7 +13515,7 @@
         <x:v>19475122.44</x:v>
       </x:c>
       <x:c r="H106" s="50" t="n">
-        <x:v>0.00002306373374345799</x:v>
+        <x:v>0.000023063655088119593</x:v>
       </x:c>
       <x:c r="I106" s="50" t="n">
         <x:v>1</x:v>

</xml_diff>